<commit_message>
feat(campaign): CLIENT-READY cycle PASS after Tiago human ACCEPT
Record explicit human acceptance (Tiago Sasaki) of the RC pack and
re-run make client-ready-consulting-cycle path. Terminal PASS with
production_touched=false, soak_touched=false, A–E + linkage + recurrence
green on isolated authenticated dump.
</commit_message>
<xml_diff>
--- a/artifacts/campaigns/CLIENT-READY-RECURRING-CONSULTING-CYCLE-01/weekly/extra_weekly_pack.xlsx
+++ b/artifacts/campaigns/CLIENT-READY-RECURRING-CONSULTING-CYCLE-01/weekly/extra_weekly_pack.xlsx
@@ -443,7 +443,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>weekly-20260724T210526Z-9c0527cd9c</t>
+          <t>weekly-20260724T214052Z-5d7fc91e7c</t>
         </is>
       </c>
     </row>
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
     </row>
@@ -467,7 +467,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-24T21:05:26Z</t>
+          <t>2026-07-24T21:40:52Z</t>
         </is>
       </c>
     </row>
@@ -479,7 +479,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>c2bef8fd928c4eca5d9f6ad8e939ee2bf74c604a</t>
+          <t>4d3cfadc19a8563317d3ddcf63ee63c4551685df</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -711,33 +711,37 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>e-evidence:11360515000119-1-000013/2026</t>
+          <t>linkage-seed:00360305000104:0</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>11360515000119-1-000013/2026</t>
+          <t>SEED-PNCP-00360305000104-0</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>11360515000119</t>
+          <t>00360305000104</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>FUNDO MUNICIPAL DE SAUDE DE SANTA TEREZINHA DO PROGRESSO</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>CEFOR</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>DF</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>AQUISIÇÃO DE LENÇÓIS E MANTAS DESTINADOS AOS LEITOS DA UNIDADE BÁSICA DE SAÚDE DO MUNICÍPIO DE SANTA TEREZINHA DO PROGRESSO/SC, VISANDO ATENDER ÀS NECESSIDADES DE ACOLHIMENTO, CONFORTO, HIGIENE E BEM-</t>
+          <t>[SNAPSHOT-SEED open] (ZMES) - CONTRATAÇÃO DE ATÉ 02 (DUAS) EMPRESAS ESPECIALIZADAS NO PLANEJAMENTO, DESENVOLVIMENTO, EXECUÇÃO, MANUTENÇÃO E MONITORAMENTO DE AMBIENTES DIGITAIS E DE SOLUÇÕES DE COMUNICAÇÃO E MARKETING DIGITAL PARA A PRESTAÇÃO DE SERVIÇOS À CAIXA</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -808,12 +812,12 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260724T210527Z-37e683b782</t>
+          <t>collect-pncp_opportunities-20260724T214053Z-f8742a1bfd</t>
         </is>
       </c>
       <c r="AH2" t="inlineStr"/>
@@ -826,7 +830,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -836,33 +840,37 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>e-evidence:07654807000197-1-000072/2026</t>
+          <t>linkage-seed:00394452000103:0</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>07654807000197-1-000072/2026</t>
+          <t>SEED-PNCP-00394452000103-0</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>07654807000197</t>
+          <t>00394452000103</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>CONSORCIO INTERMUNICIPAL DE SAUDE DO ALTO URUGUAI CATARINENSE</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>SECRETARIA GERAL DO EXERCITO/MEX/DF</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Vila Velha</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>TO</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Aquisição de 01 (um) computador do tipo All in One, novo, de primeiro uso, contemplando, no mínimo, processador Intel Core i5- 12400 ou equivalente em desempenho ou superior, 16 GB de memória RAM DDR4</t>
+          <t>[SNAPSHOT-SEED open] НHOSPITAL GERAL DE MÉDIA E ALTA COMPLEXIDADE COM ATENDIMENTO AMBULATORIAL, INTERNAÇÃO E SADT.</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -933,12 +941,12 @@
       </c>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260724T210527Z-37e683b782</t>
+          <t>collect-pncp_opportunities-20260724T214053Z-f8742a1bfd</t>
         </is>
       </c>
       <c r="AH3" t="inlineStr"/>
@@ -951,7 +959,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -961,33 +969,37 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>e-evidence:10432684000154-1-000049/2025</t>
+          <t>linkage-seed:00394544000185:0</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10432684000154-1-000049/2025</t>
+          <t>SEED-PNCP-00394544000185-0</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10432684000154</t>
+          <t>00394544000185</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>FUNDO MUNICIPAL DE SAUDE</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>SUPERINTENDENCIA ESTADUAL DO MS/TO</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>TO</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>CREDENCIAMENTO DE EMPRESA ESPECIALIZADA PARA EXECUÇÃO DE SERVIÇOS DE FORMA COMPLEMENTAR AO SUS, DE EXAMES COM FINALIDADE DIAGNÓSTICA (LABORATÓRIO CLÍNICO), EXAMES BIOQUÍMICOS, HEMATOLÓGICOS E HEMOSTAS</t>
+          <t>[SNAPSHOT-SEED open] VISTO À AQUISIÇÃO EMERGENCIAL DE EQUIPAMENTOS NÁUTICOS PARA ATENDER ÀS NECESSIDADES DA CASAI DE GUAJARÁ-MIRIM/RO, MOTOR DE POPA 150HP 4 TEMPOS MARCA MERCURY MODELO 150L EFI 4STK SEA PRO ALTERNADOR A/W 60 AMP 756 WATTS .25061.001959/2025-35.</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
@@ -1058,12 +1070,12 @@
       </c>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260724T210527Z-37e683b782</t>
+          <t>collect-pncp_opportunities-20260724T214053Z-f8742a1bfd</t>
         </is>
       </c>
       <c r="AH4" t="inlineStr"/>
@@ -1076,7 +1088,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1086,22 +1098,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>e-evidence:83102541000158-1-000167/2025</t>
+          <t>e-evidence:11360515000119-1-000013/2026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>83102541000158-1-000167/2025</t>
+          <t>11360515000119-1-000013/2026</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>83102541000158</t>
+          <t>11360515000119</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE PORTO UNIAO</t>
+          <t>FUNDO MUNICIPAL DE SAUDE DE SANTA TEREZINHA DO PROGRESSO</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -1112,7 +1124,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Credenciamento de empresa para prestação de serviços de manutenção da frota municipal, incluindo fornecimento de peças e serviços necessários, visando à aquisição de serviços de manutenção mecânica, e</t>
+          <t>AQUISIÇÃO DE LENÇÓIS E MANTAS DESTINADOS AOS LEITOS DA UNIDADE BÁSICA DE SAÚDE DO MUNICÍPIO DE SANTA TEREZINHA DO PROGRESSO/SC, VISANDO ATENDER ÀS NECESSIDADES DE ACOLHIMENTO, CONFORTO, HIGIENE E BEM-</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
@@ -1157,7 +1169,7 @@
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>2026-07-24 21:04:54.438026+00:00</t>
+          <t>2026-07-24 21:40:22.770687+00:00</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
@@ -1183,12 +1195,12 @@
       </c>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260724T210527Z-37e683b782</t>
+          <t>collect-pncp_opportunities-20260724T214053Z-f8742a1bfd</t>
         </is>
       </c>
       <c r="AH5" t="inlineStr"/>
@@ -1201,7 +1213,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1211,37 +1223,33 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>linkage-seed:00360305000104:0</t>
+          <t>e-evidence:07654807000197-1-000072/2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>SEED-PNCP-00360305000104-0</t>
+          <t>07654807000197-1-000072/2026</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>00360305000104</t>
+          <t>07654807000197</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>CEFOR</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Brasília</t>
-        </is>
-      </c>
+          <t>CONSORCIO INTERMUNICIPAL DE SAUDE DO ALTO URUGUAI CATARINENSE</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>DF</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>[SNAPSHOT-SEED open] (ZMES) - CONTRATAÇÃO DE ATÉ 02 (DUAS) EMPRESAS ESPECIALIZADAS NO PLANEJAMENTO, DESENVOLVIMENTO, EXECUÇÃO, MANUTENÇÃO E MONITORAMENTO DE AMBIENTES DIGITAIS E DE SOLUÇÕES DE COMUNICAÇÃO E MARKETING DIGITAL PARA A PRESTAÇÃO DE SERVIÇOS À CAIXA</t>
+          <t>Aquisição de 01 (um) computador do tipo All in One, novo, de primeiro uso, contemplando, no mínimo, processador Intel Core i5- 12400 ou equivalente em desempenho ou superior, 16 GB de memória RAM DDR4</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
@@ -1286,7 +1294,7 @@
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>2026-07-24 21:04:54.438026+00:00</t>
+          <t>2026-07-24 21:40:22.770687+00:00</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
@@ -1312,12 +1320,12 @@
       </c>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260724T210527Z-37e683b782</t>
+          <t>collect-pncp_opportunities-20260724T214053Z-f8742a1bfd</t>
         </is>
       </c>
       <c r="AH6" t="inlineStr"/>
@@ -1330,7 +1338,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1340,37 +1348,33 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>linkage-seed:00394452000103:0</t>
+          <t>e-evidence:10432684000154-1-000049/2025</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>SEED-PNCP-00394452000103-0</t>
+          <t>10432684000154-1-000049/2025</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>00394452000103</t>
+          <t>10432684000154</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>SECRETARIA GERAL DO EXERCITO/MEX/DF</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Vila Velha</t>
-        </is>
-      </c>
+          <t>FUNDO MUNICIPAL DE SAUDE</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>[SNAPSHOT-SEED open] НHOSPITAL GERAL DE MÉDIA E ALTA COMPLEXIDADE COM ATENDIMENTO AMBULATORIAL, INTERNAÇÃO E SADT.</t>
+          <t>CREDENCIAMENTO DE EMPRESA ESPECIALIZADA PARA EXECUÇÃO DE SERVIÇOS DE FORMA COMPLEMENTAR AO SUS, DE EXAMES COM FINALIDADE DIAGNÓSTICA (LABORATÓRIO CLÍNICO), EXAMES BIOQUÍMICOS, HEMATOLÓGICOS E HEMOSTAS</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
@@ -1415,7 +1419,7 @@
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>2026-07-24 21:04:54.438026+00:00</t>
+          <t>2026-07-24 21:40:22.770687+00:00</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr">
@@ -1441,12 +1445,12 @@
       </c>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260724T210527Z-37e683b782</t>
+          <t>collect-pncp_opportunities-20260724T214053Z-f8742a1bfd</t>
         </is>
       </c>
       <c r="AH7" t="inlineStr"/>
@@ -1459,7 +1463,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1469,37 +1473,33 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>linkage-seed:00394544000185:0</t>
+          <t>e-evidence:83102541000158-1-000167/2025</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>SEED-PNCP-00394544000185-0</t>
+          <t>83102541000158-1-000167/2025</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>00394544000185</t>
+          <t>83102541000158</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>SUPERINTENDENCIA ESTADUAL DO MS/TO</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Vitória</t>
-        </is>
-      </c>
+          <t>MUNICIPIO DE PORTO UNIAO</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>[SNAPSHOT-SEED open] VISTO À AQUISIÇÃO EMERGENCIAL DE EQUIPAMENTOS NÁUTICOS PARA ATENDER ÀS NECESSIDADES DA CASAI DE GUAJARÁ-MIRIM/RO, MOTOR DE POPA 150HP 4 TEMPOS MARCA MERCURY MODELO 150L EFI 4STK SEA PRO ALTERNADOR A/W 60 AMP 756 WATTS .25061.001959/2025-35.</t>
+          <t>Credenciamento de empresa para prestação de serviços de manutenção da frota municipal, incluindo fornecimento de peças e serviços necessários, visando à aquisição de serviços de manutenção mecânica, e</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
@@ -1544,7 +1544,7 @@
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>2026-07-24 21:04:54.438026+00:00</t>
+          <t>2026-07-24 21:40:22.770687+00:00</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr">
@@ -1570,12 +1570,12 @@
       </c>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260724T210527Z-37e683b782</t>
+          <t>collect-pncp_opportunities-20260724T214053Z-f8742a1bfd</t>
         </is>
       </c>
       <c r="AH8" t="inlineStr"/>
@@ -1834,12 +1834,12 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W2" t="inlineStr"/>
@@ -1962,12 +1962,12 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W3" t="inlineStr"/>
@@ -2090,12 +2090,12 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W4" t="inlineStr"/>
@@ -2218,12 +2218,12 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W5" t="inlineStr"/>
@@ -2346,12 +2346,12 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W6" t="inlineStr"/>
@@ -2474,12 +2474,12 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W7" t="inlineStr"/>
@@ -2602,12 +2602,12 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W8" t="inlineStr"/>
@@ -2730,12 +2730,12 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W9" t="inlineStr"/>
@@ -2858,12 +2858,12 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W10" t="inlineStr"/>
@@ -2986,12 +2986,12 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W11" t="inlineStr"/>
@@ -3114,12 +3114,12 @@
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W12" t="inlineStr"/>
@@ -3242,12 +3242,12 @@
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W13" t="inlineStr"/>
@@ -3370,12 +3370,12 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W14" t="inlineStr"/>
@@ -3498,12 +3498,12 @@
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W15" t="inlineStr"/>
@@ -3626,12 +3626,12 @@
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W16" t="inlineStr"/>
@@ -3754,12 +3754,12 @@
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W17" t="inlineStr"/>
@@ -3882,12 +3882,12 @@
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W18" t="inlineStr"/>
@@ -4010,12 +4010,12 @@
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W19" t="inlineStr"/>
@@ -4138,12 +4138,12 @@
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W20" t="inlineStr"/>
@@ -4266,12 +4266,12 @@
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W21" t="inlineStr"/>
@@ -4394,12 +4394,12 @@
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W22" t="inlineStr"/>
@@ -4522,12 +4522,12 @@
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W23" t="inlineStr"/>
@@ -4650,12 +4650,12 @@
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W24" t="inlineStr"/>
@@ -4778,12 +4778,12 @@
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W25" t="inlineStr"/>
@@ -4906,12 +4906,12 @@
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W26" t="inlineStr"/>
@@ -5034,12 +5034,12 @@
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W27" t="inlineStr"/>
@@ -5162,12 +5162,12 @@
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W28" t="inlineStr"/>
@@ -5290,12 +5290,12 @@
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W29" t="inlineStr"/>
@@ -5418,12 +5418,12 @@
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W30" t="inlineStr"/>
@@ -5546,12 +5546,12 @@
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="W31" t="inlineStr"/>
@@ -5680,12 +5680,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -5737,12 +5737,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -5794,12 +5794,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -5851,12 +5851,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -5908,12 +5908,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -5965,12 +5965,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -6022,12 +6022,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -6079,12 +6079,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -6136,12 +6136,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -6193,12 +6193,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -6250,12 +6250,12 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -6307,12 +6307,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -6364,12 +6364,12 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -6421,12 +6421,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -6478,12 +6478,12 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -6535,12 +6535,12 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -6592,12 +6592,12 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -6649,12 +6649,12 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -6706,12 +6706,12 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -6763,12 +6763,12 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -6820,12 +6820,12 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -6877,12 +6877,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -6934,12 +6934,12 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -6991,12 +6991,12 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -7048,12 +7048,12 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -7105,12 +7105,12 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -7162,12 +7162,12 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -7219,12 +7219,12 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -7276,12 +7276,12 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -7333,12 +7333,12 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T210528Z-d81cfd4c1f</t>
+          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -7431,7 +7431,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -7505,7 +7505,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -7538,7 +7538,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -7571,7 +7571,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -7604,7 +7604,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -7637,7 +7637,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T210526Z-b2b865fa</t>
+          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -7728,7 +7728,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>25.27</t>
+          <t>25.86</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">

</xml_diff>

<commit_message>
fix(campaign): honest labeled recurrence; pack cut consistency; skeptic gaps
- Label monthly two-cycle as LABELED_DETERMINISTIC_REPLAY (same snapshot +
  inject); never claim live_dual_snapshot for synthetic LIVE-DELTA/SUSPENSAO.
- decide_terminal FAILs false live_dual claims; PASS allowed with human ACCEPT
  + mechanics proven without dual temporal exports.
- Always overwrite pack aliases so executive-summary/meeting-support share run_id.
- Bind acceptance package_checksums to full pack tree; populate manifest
  snapshot_sha256 (SHA256SUMS), gate_results, ci_run.
- Re-run cycle: PASS with consistent run_id and zero checksum mismatches.
</commit_message>
<xml_diff>
--- a/artifacts/campaigns/CLIENT-READY-RECURRING-CONSULTING-CYCLE-01/weekly/extra_weekly_pack.xlsx
+++ b/artifacts/campaigns/CLIENT-READY-RECURRING-CONSULTING-CYCLE-01/weekly/extra_weekly_pack.xlsx
@@ -443,7 +443,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>weekly-20260724T214052Z-5d7fc91e7c</t>
+          <t>weekly-20260724T215115Z-6d643e108f</t>
         </is>
       </c>
     </row>
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
     </row>
@@ -467,7 +467,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-24T21:40:52Z</t>
+          <t>2026-07-24T21:51:16Z</t>
         </is>
       </c>
     </row>
@@ -479,7 +479,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>4d3cfadc19a8563317d3ddcf63ee63c4551685df</t>
+          <t>9662ce478bde3345297711746b6ecfe225564dd7</t>
         </is>
       </c>
     </row>
@@ -812,12 +812,12 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260724T214053Z-f8742a1bfd</t>
+          <t>collect-pncp_opportunities-20260724T215117Z-ad4de2a078</t>
         </is>
       </c>
       <c r="AH2" t="inlineStr"/>
@@ -941,12 +941,12 @@
       </c>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260724T214053Z-f8742a1bfd</t>
+          <t>collect-pncp_opportunities-20260724T215117Z-ad4de2a078</t>
         </is>
       </c>
       <c r="AH3" t="inlineStr"/>
@@ -1070,12 +1070,12 @@
       </c>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260724T214053Z-f8742a1bfd</t>
+          <t>collect-pncp_opportunities-20260724T215117Z-ad4de2a078</t>
         </is>
       </c>
       <c r="AH4" t="inlineStr"/>
@@ -1169,7 +1169,7 @@
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>2026-07-24 21:40:22.770687+00:00</t>
+          <t>2026-07-24 21:50:50.296555+00:00</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
@@ -1195,12 +1195,12 @@
       </c>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260724T214053Z-f8742a1bfd</t>
+          <t>collect-pncp_opportunities-20260724T215117Z-ad4de2a078</t>
         </is>
       </c>
       <c r="AH5" t="inlineStr"/>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>2026-07-24 21:40:22.770687+00:00</t>
+          <t>2026-07-24 21:50:50.296555+00:00</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
@@ -1320,12 +1320,12 @@
       </c>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260724T214053Z-f8742a1bfd</t>
+          <t>collect-pncp_opportunities-20260724T215117Z-ad4de2a078</t>
         </is>
       </c>
       <c r="AH6" t="inlineStr"/>
@@ -1419,7 +1419,7 @@
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>2026-07-24 21:40:22.770687+00:00</t>
+          <t>2026-07-24 21:50:50.296555+00:00</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr">
@@ -1445,12 +1445,12 @@
       </c>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260724T214053Z-f8742a1bfd</t>
+          <t>collect-pncp_opportunities-20260724T215117Z-ad4de2a078</t>
         </is>
       </c>
       <c r="AH7" t="inlineStr"/>
@@ -1544,7 +1544,7 @@
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>2026-07-24 21:40:22.770687+00:00</t>
+          <t>2026-07-24 21:50:50.296555+00:00</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr">
@@ -1570,12 +1570,12 @@
       </c>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260724T214053Z-f8742a1bfd</t>
+          <t>collect-pncp_opportunities-20260724T215117Z-ad4de2a078</t>
         </is>
       </c>
       <c r="AH8" t="inlineStr"/>
@@ -1834,12 +1834,12 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W2" t="inlineStr"/>
@@ -1962,12 +1962,12 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W3" t="inlineStr"/>
@@ -2090,12 +2090,12 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W4" t="inlineStr"/>
@@ -2218,12 +2218,12 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W5" t="inlineStr"/>
@@ -2346,12 +2346,12 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W6" t="inlineStr"/>
@@ -2474,12 +2474,12 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W7" t="inlineStr"/>
@@ -2602,12 +2602,12 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W8" t="inlineStr"/>
@@ -2730,12 +2730,12 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W9" t="inlineStr"/>
@@ -2858,12 +2858,12 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W10" t="inlineStr"/>
@@ -2986,12 +2986,12 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W11" t="inlineStr"/>
@@ -3114,12 +3114,12 @@
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W12" t="inlineStr"/>
@@ -3242,12 +3242,12 @@
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W13" t="inlineStr"/>
@@ -3370,12 +3370,12 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W14" t="inlineStr"/>
@@ -3498,12 +3498,12 @@
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W15" t="inlineStr"/>
@@ -3626,12 +3626,12 @@
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W16" t="inlineStr"/>
@@ -3754,12 +3754,12 @@
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W17" t="inlineStr"/>
@@ -3882,12 +3882,12 @@
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W18" t="inlineStr"/>
@@ -4010,12 +4010,12 @@
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W19" t="inlineStr"/>
@@ -4138,12 +4138,12 @@
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W20" t="inlineStr"/>
@@ -4266,12 +4266,12 @@
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W21" t="inlineStr"/>
@@ -4394,12 +4394,12 @@
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W22" t="inlineStr"/>
@@ -4522,12 +4522,12 @@
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W23" t="inlineStr"/>
@@ -4650,12 +4650,12 @@
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W24" t="inlineStr"/>
@@ -4778,12 +4778,12 @@
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W25" t="inlineStr"/>
@@ -4906,12 +4906,12 @@
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W26" t="inlineStr"/>
@@ -5034,12 +5034,12 @@
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W27" t="inlineStr"/>
@@ -5162,12 +5162,12 @@
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W28" t="inlineStr"/>
@@ -5290,12 +5290,12 @@
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W29" t="inlineStr"/>
@@ -5418,12 +5418,12 @@
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W30" t="inlineStr"/>
@@ -5546,12 +5546,12 @@
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="W31" t="inlineStr"/>
@@ -5680,12 +5680,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -5737,12 +5737,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -5794,12 +5794,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -5851,12 +5851,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -5908,12 +5908,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -5965,12 +5965,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -6022,12 +6022,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -6079,12 +6079,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -6136,12 +6136,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -6193,12 +6193,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -6250,12 +6250,12 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -6307,12 +6307,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -6364,12 +6364,12 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -6421,12 +6421,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -6478,12 +6478,12 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -6535,12 +6535,12 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -6592,12 +6592,12 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -6649,12 +6649,12 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -6706,12 +6706,12 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -6763,12 +6763,12 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -6820,12 +6820,12 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -6877,12 +6877,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -6934,12 +6934,12 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -6991,12 +6991,12 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -7048,12 +7048,12 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -7105,12 +7105,12 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -7162,12 +7162,12 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -7219,12 +7219,12 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -7276,12 +7276,12 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -7333,12 +7333,12 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T214053Z-978b39a746</t>
+          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -7431,7 +7431,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -7505,7 +7505,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -7538,7 +7538,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -7571,7 +7571,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -7604,7 +7604,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -7637,7 +7637,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T214052Z-8da20af7</t>
+          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -7728,7 +7728,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>25.86</t>
+          <t>26.04</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">

</xml_diff>

<commit_message>
docs(campaign): freeze RC pack after accept-binding fix (PENDING_HUMAN)
Stale ACCEPT demoted; pack run_id/rc_sha/checksums ready for re-accept
bound to this release candidate only. Labeled recurrence non-claim holds.
</commit_message>
<xml_diff>
--- a/artifacts/campaigns/CLIENT-READY-RECURRING-CONSULTING-CYCLE-01/weekly/extra_weekly_pack.xlsx
+++ b/artifacts/campaigns/CLIENT-READY-RECURRING-CONSULTING-CYCLE-01/weekly/extra_weekly_pack.xlsx
@@ -443,7 +443,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>weekly-20260724T215115Z-6d643e108f</t>
+          <t>weekly-20260724T220411Z-29c46fab61</t>
         </is>
       </c>
     </row>
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
     </row>
@@ -467,7 +467,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-24T21:51:16Z</t>
+          <t>2026-07-24T22:04:11Z</t>
         </is>
       </c>
     </row>
@@ -479,7 +479,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>9662ce478bde3345297711746b6ecfe225564dd7</t>
+          <t>be96c8bc8eb2b017e491bfafe8cf99f81e321267</t>
         </is>
       </c>
     </row>
@@ -812,12 +812,12 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260724T215117Z-ad4de2a078</t>
+          <t>collect-pncp_opportunities-20260724T220412Z-6051e30a5a</t>
         </is>
       </c>
       <c r="AH2" t="inlineStr"/>
@@ -941,12 +941,12 @@
       </c>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260724T215117Z-ad4de2a078</t>
+          <t>collect-pncp_opportunities-20260724T220412Z-6051e30a5a</t>
         </is>
       </c>
       <c r="AH3" t="inlineStr"/>
@@ -1070,12 +1070,12 @@
       </c>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260724T215117Z-ad4de2a078</t>
+          <t>collect-pncp_opportunities-20260724T220412Z-6051e30a5a</t>
         </is>
       </c>
       <c r="AH4" t="inlineStr"/>
@@ -1169,7 +1169,7 @@
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>2026-07-24 21:50:50.296555+00:00</t>
+          <t>2026-07-24 22:03:45.267218+00:00</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
@@ -1195,12 +1195,12 @@
       </c>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260724T215117Z-ad4de2a078</t>
+          <t>collect-pncp_opportunities-20260724T220412Z-6051e30a5a</t>
         </is>
       </c>
       <c r="AH5" t="inlineStr"/>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>2026-07-24 21:50:50.296555+00:00</t>
+          <t>2026-07-24 22:03:45.267218+00:00</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
@@ -1320,12 +1320,12 @@
       </c>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260724T215117Z-ad4de2a078</t>
+          <t>collect-pncp_opportunities-20260724T220412Z-6051e30a5a</t>
         </is>
       </c>
       <c r="AH6" t="inlineStr"/>
@@ -1419,7 +1419,7 @@
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>2026-07-24 21:50:50.296555+00:00</t>
+          <t>2026-07-24 22:03:45.267218+00:00</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr">
@@ -1445,12 +1445,12 @@
       </c>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260724T215117Z-ad4de2a078</t>
+          <t>collect-pncp_opportunities-20260724T220412Z-6051e30a5a</t>
         </is>
       </c>
       <c r="AH7" t="inlineStr"/>
@@ -1544,7 +1544,7 @@
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>2026-07-24 21:50:50.296555+00:00</t>
+          <t>2026-07-24 22:03:45.267218+00:00</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr">
@@ -1570,12 +1570,12 @@
       </c>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>collect-pncp_opportunities-20260724T215117Z-ad4de2a078</t>
+          <t>collect-pncp_opportunities-20260724T220412Z-6051e30a5a</t>
         </is>
       </c>
       <c r="AH8" t="inlineStr"/>
@@ -1834,12 +1834,12 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W2" t="inlineStr"/>
@@ -1962,12 +1962,12 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W3" t="inlineStr"/>
@@ -2090,12 +2090,12 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W4" t="inlineStr"/>
@@ -2218,12 +2218,12 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W5" t="inlineStr"/>
@@ -2346,12 +2346,12 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W6" t="inlineStr"/>
@@ -2474,12 +2474,12 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W7" t="inlineStr"/>
@@ -2602,12 +2602,12 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W8" t="inlineStr"/>
@@ -2730,12 +2730,12 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W9" t="inlineStr"/>
@@ -2858,12 +2858,12 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W10" t="inlineStr"/>
@@ -2986,12 +2986,12 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W11" t="inlineStr"/>
@@ -3114,12 +3114,12 @@
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W12" t="inlineStr"/>
@@ -3242,12 +3242,12 @@
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W13" t="inlineStr"/>
@@ -3370,12 +3370,12 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W14" t="inlineStr"/>
@@ -3498,12 +3498,12 @@
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W15" t="inlineStr"/>
@@ -3626,12 +3626,12 @@
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W16" t="inlineStr"/>
@@ -3754,12 +3754,12 @@
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W17" t="inlineStr"/>
@@ -3882,12 +3882,12 @@
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W18" t="inlineStr"/>
@@ -4010,12 +4010,12 @@
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W19" t="inlineStr"/>
@@ -4138,12 +4138,12 @@
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W20" t="inlineStr"/>
@@ -4266,12 +4266,12 @@
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W21" t="inlineStr"/>
@@ -4394,12 +4394,12 @@
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W22" t="inlineStr"/>
@@ -4522,12 +4522,12 @@
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W23" t="inlineStr"/>
@@ -4650,12 +4650,12 @@
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W24" t="inlineStr"/>
@@ -4778,12 +4778,12 @@
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W25" t="inlineStr"/>
@@ -4906,12 +4906,12 @@
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W26" t="inlineStr"/>
@@ -5034,12 +5034,12 @@
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W27" t="inlineStr"/>
@@ -5162,12 +5162,12 @@
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W28" t="inlineStr"/>
@@ -5290,12 +5290,12 @@
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W29" t="inlineStr"/>
@@ -5418,12 +5418,12 @@
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W30" t="inlineStr"/>
@@ -5546,12 +5546,12 @@
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="W31" t="inlineStr"/>
@@ -5680,12 +5680,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -5737,12 +5737,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -5794,12 +5794,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -5851,12 +5851,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -5908,12 +5908,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -5965,12 +5965,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -6022,12 +6022,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -6079,12 +6079,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -6136,12 +6136,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -6193,12 +6193,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -6250,12 +6250,12 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -6307,12 +6307,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -6364,12 +6364,12 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -6421,12 +6421,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -6478,12 +6478,12 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -6535,12 +6535,12 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -6592,12 +6592,12 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -6649,12 +6649,12 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -6706,12 +6706,12 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -6763,12 +6763,12 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -6820,12 +6820,12 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -6877,12 +6877,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -6934,12 +6934,12 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -6991,12 +6991,12 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -7048,12 +7048,12 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -7105,12 +7105,12 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -7162,12 +7162,12 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -7219,12 +7219,12 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -7276,12 +7276,12 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -7333,12 +7333,12 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>collect-pncp_contracts-20260724T215117Z-ebf6e0d883</t>
+          <t>collect-pncp_contracts-20260724T220413Z-d4f8aa5d3b</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -7431,7 +7431,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -7505,7 +7505,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -7538,7 +7538,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -7571,7 +7571,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -7604,7 +7604,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -7637,7 +7637,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>col-extra-weekly-20260724T215115Z-178bc934</t>
+          <t>col-extra-weekly-20260724T220411Z-71efe758</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -7728,7 +7728,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>26.04</t>
+          <t>26.25</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">

</xml_diff>